<commit_message>
Add minimal data model for regulatory GA structure (schema only)
Adds plant_code/fiscal_year/industry_type/company_size to 30_contract.xlsx,
supply_type to 22_material_issue.xlsx (and its byte-identical duplicate
fixture), and a headers-only 32_cost_rate_rule.xlsx, plus a new
calculate_government_furnished_material_by_contract() combine-function.
No real GA rate/GFM values are populated and no existing function or the
CLI is touched — this only prepares the data model for the regulation-
compliant GA path built in prior rounds.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hanbit_mvp_dataset_phase1/22_material_issue.xlsx
+++ b/hanbit_mvp_dataset_phase1/22_material_issue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="material_issue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="material_issue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'material_issue'!$A$1:$I$63</definedName>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,6 +471,11 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>issue_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>supply_type</t>
         </is>
       </c>
     </row>

</xml_diff>